<commit_message>
Modification tableau synthèse compétences
</commit_message>
<xml_diff>
--- a/Tableau_synthese_ALMAZAN-LAFORET_Hugo_2026.xlsx
+++ b/Tableau_synthese_ALMAZAN-LAFORET_Hugo_2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hugo\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A4F9A8B-8342-4978-94A7-3FD880638099}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{775E2871-40D3-4561-8EAC-1482108E01FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Tableau de synthèse Épreuve E5" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau de synthèse Épreuve E5'!$A$1:$H$24</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau de synthèse Épreuve E5'!$A$1:$H$26</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -151,12 +151,6 @@
 pour suivi des VCS</t>
   </si>
   <si>
-    <t>BeSafe: Application web permettant de gérer les visites comportementales de sécurité</t>
-  </si>
-  <si>
-    <t>Klimarine: Application web pour laquage dans la chaine de production</t>
-  </si>
-  <si>
     <t>01/01/2026
 au
 ?</t>
@@ -167,14 +161,22 @@
 ?</t>
   </si>
   <si>
-    <t>26/05/2025 
+    <t>Klimarine: Application web pour gestion qualimarine pour laquage dans la chaine
+de production</t>
+  </si>
+  <si>
+    <t>26/05/2025
 au
 04/07/2025</t>
   </si>
   <si>
-    <t>04/07/2025
-au
-26/08/2025</t>
+    <t>07/07/2025
+au 
+28/08/2025</t>
+  </si>
+  <si>
+    <t>BeSafe: Application web permettant de gérer les visites comportementales
+de sécurité (VCS)</t>
   </si>
 </sst>
 </file>
@@ -775,7 +777,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -813,6 +815,63 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -876,13 +935,37 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -891,58 +974,10 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="9" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1178,67 +1213,66 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AQ81"/>
+  <dimension ref="A1:AH83"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.85546875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="70.42578125" style="1" customWidth="1"/>
     <col min="2" max="2" width="19.7109375" style="1" customWidth="1"/>
     <col min="3" max="8" width="18.7109375" style="1" customWidth="1"/>
-    <col min="9" max="43" width="11.42578125" customWidth="1"/>
-    <col min="44" max="16384" width="10.85546875" style="1"/>
+    <col min="9" max="34" width="11.42578125" customWidth="1"/>
+    <col min="35" max="16384" width="10.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="13" t="s">
+    <row r="1" spans="1:34" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13" t="s">
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="13"/>
-    </row>
-    <row r="2" spans="1:43" ht="41.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="13" t="s">
+      <c r="H1" s="32"/>
+    </row>
+    <row r="2" spans="1:34" ht="41.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13"/>
-      <c r="H2" s="13"/>
-    </row>
-    <row r="3" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="14" t="s">
+      <c r="B2" s="32"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="32"/>
+    </row>
+    <row r="3" spans="1:34" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="B3" s="15"/>
-      <c r="C3" s="15"/>
-      <c r="D3" s="15"/>
-      <c r="E3" s="16"/>
-      <c r="F3" s="17" t="s">
+      <c r="B3" s="34"/>
+      <c r="C3" s="34"/>
+      <c r="D3" s="34"/>
+      <c r="E3" s="35"/>
+      <c r="F3" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="15"/>
-      <c r="H3" s="18"/>
+      <c r="G3" s="34"/>
+      <c r="H3" s="37"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
-      <c r="M3" s="1"/>
-    </row>
-    <row r="4" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="22" t="s">
+    </row>
+    <row r="4" spans="1:34" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="B4" s="23"/>
-      <c r="C4" s="23"/>
-      <c r="D4" s="23"/>
-      <c r="E4" s="24"/>
+      <c r="B4" s="42"/>
+      <c r="C4" s="42"/>
+      <c r="D4" s="42"/>
+      <c r="E4" s="43"/>
       <c r="F4" s="2" t="s">
         <v>4</v>
       </c>
@@ -1249,23 +1283,23 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="25" t="s">
+    <row r="5" spans="1:34" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="44" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="26"/>
-      <c r="C5" s="26"/>
-      <c r="D5" s="26"/>
-      <c r="E5" s="26"/>
-      <c r="F5" s="26"/>
-      <c r="G5" s="26"/>
-      <c r="H5" s="27"/>
-    </row>
-    <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="28" t="s">
+      <c r="B5" s="45"/>
+      <c r="C5" s="45"/>
+      <c r="D5" s="45"/>
+      <c r="E5" s="45"/>
+      <c r="F5" s="45"/>
+      <c r="G5" s="45"/>
+      <c r="H5" s="46"/>
+    </row>
+    <row r="6" spans="1:34" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="47" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="30" t="s">
+      <c r="B6" s="49" t="s">
         <v>7</v>
       </c>
       <c r="C6" s="5" t="s">
@@ -1287,9 +1321,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:43" s="7" customFormat="1" ht="324.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="29"/>
-      <c r="B7" s="31"/>
+    <row r="7" spans="1:34" s="7" customFormat="1" ht="324.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="48"/>
+      <c r="B7" s="50"/>
       <c r="C7" s="8" t="s">
         <v>14</v>
       </c>
@@ -1334,27 +1368,18 @@
       <c r="AF7"/>
       <c r="AG7"/>
       <c r="AH7"/>
-      <c r="AI7"/>
-      <c r="AJ7"/>
-      <c r="AK7"/>
-      <c r="AL7"/>
-      <c r="AM7"/>
-      <c r="AN7"/>
-      <c r="AO7"/>
-      <c r="AP7"/>
-      <c r="AQ7"/>
-    </row>
-    <row r="8" spans="1:43" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A8" s="32" t="s">
+    </row>
+    <row r="8" spans="1:34" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.2">
+      <c r="A8" s="51" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="33"/>
-      <c r="C8" s="33"/>
-      <c r="D8" s="39"/>
-      <c r="E8" s="39"/>
-      <c r="F8" s="39"/>
-      <c r="G8" s="39"/>
-      <c r="H8" s="40"/>
+      <c r="B8" s="52"/>
+      <c r="C8" s="52"/>
+      <c r="D8" s="53"/>
+      <c r="E8" s="53"/>
+      <c r="F8" s="53"/>
+      <c r="G8" s="53"/>
+      <c r="H8" s="54"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1381,29 +1406,20 @@
       <c r="AF8"/>
       <c r="AG8"/>
       <c r="AH8"/>
-      <c r="AI8"/>
-      <c r="AJ8"/>
-      <c r="AK8"/>
-      <c r="AL8"/>
-      <c r="AM8"/>
-      <c r="AN8"/>
-      <c r="AO8"/>
-      <c r="AP8"/>
-      <c r="AQ8"/>
-    </row>
-    <row r="9" spans="1:43" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="37" t="s">
+    </row>
+    <row r="9" spans="1:34" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="64" t="s">
         <v>27</v>
       </c>
-      <c r="B9" s="46" t="s">
-        <v>32</v>
-      </c>
-      <c r="C9" s="41"/>
-      <c r="D9" s="49"/>
-      <c r="E9" s="43"/>
-      <c r="F9" s="43"/>
-      <c r="G9" s="43"/>
-      <c r="H9" s="43"/>
+      <c r="B9" s="60" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" s="62"/>
+      <c r="D9" s="66"/>
+      <c r="E9" s="55"/>
+      <c r="F9" s="55"/>
+      <c r="G9" s="55"/>
+      <c r="H9" s="55"/>
       <c r="I9"/>
       <c r="J9"/>
       <c r="K9"/>
@@ -1430,25 +1446,16 @@
       <c r="AF9"/>
       <c r="AG9"/>
       <c r="AH9"/>
-      <c r="AI9"/>
-      <c r="AJ9"/>
-      <c r="AK9"/>
-      <c r="AL9"/>
-      <c r="AM9"/>
-      <c r="AN9"/>
-      <c r="AO9"/>
-      <c r="AP9"/>
-      <c r="AQ9"/>
-    </row>
-    <row r="10" spans="1:43" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="38"/>
-      <c r="B10" s="47"/>
-      <c r="C10" s="42"/>
-      <c r="D10" s="50"/>
-      <c r="E10" s="44"/>
-      <c r="F10" s="44"/>
-      <c r="G10" s="44"/>
-      <c r="H10" s="44"/>
+    </row>
+    <row r="10" spans="1:34" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="65"/>
+      <c r="B10" s="61"/>
+      <c r="C10" s="63"/>
+      <c r="D10" s="67"/>
+      <c r="E10" s="56"/>
+      <c r="F10" s="56"/>
+      <c r="G10" s="56"/>
+      <c r="H10" s="56"/>
       <c r="I10"/>
       <c r="J10"/>
       <c r="K10"/>
@@ -1475,29 +1482,20 @@
       <c r="AF10"/>
       <c r="AG10"/>
       <c r="AH10"/>
-      <c r="AI10"/>
-      <c r="AJ10"/>
-      <c r="AK10"/>
-      <c r="AL10"/>
-      <c r="AM10"/>
-      <c r="AN10"/>
-      <c r="AO10"/>
-      <c r="AP10"/>
-      <c r="AQ10"/>
-    </row>
-    <row r="11" spans="1:43" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="34" t="s">
+    </row>
+    <row r="11" spans="1:34" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="B11" s="45" t="s">
-        <v>32</v>
-      </c>
-      <c r="C11" s="51"/>
-      <c r="D11" s="52"/>
-      <c r="E11" s="52"/>
-      <c r="F11" s="52"/>
-      <c r="G11" s="52"/>
-      <c r="H11" s="53"/>
+      <c r="B11" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="C11" s="15"/>
+      <c r="D11" s="58"/>
+      <c r="E11" s="58"/>
+      <c r="F11" s="58"/>
+      <c r="G11" s="58"/>
+      <c r="H11" s="59"/>
       <c r="I11"/>
       <c r="J11"/>
       <c r="K11"/>
@@ -1524,25 +1522,16 @@
       <c r="AF11"/>
       <c r="AG11"/>
       <c r="AH11"/>
-      <c r="AI11"/>
-      <c r="AJ11"/>
-      <c r="AK11"/>
-      <c r="AL11"/>
-      <c r="AM11"/>
-      <c r="AN11"/>
-      <c r="AO11"/>
-      <c r="AP11"/>
-      <c r="AQ11"/>
-    </row>
-    <row r="12" spans="1:43" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="35"/>
-      <c r="B12" s="36"/>
-      <c r="C12" s="54"/>
-      <c r="D12" s="54"/>
-      <c r="E12" s="54"/>
-      <c r="F12" s="54"/>
-      <c r="G12" s="54"/>
-      <c r="H12" s="55"/>
+    </row>
+    <row r="12" spans="1:34" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="20"/>
+      <c r="B12" s="57"/>
+      <c r="C12" s="16"/>
+      <c r="D12" s="16"/>
+      <c r="E12" s="16"/>
+      <c r="F12" s="16"/>
+      <c r="G12" s="16"/>
+      <c r="H12" s="31"/>
       <c r="I12"/>
       <c r="J12"/>
       <c r="K12"/>
@@ -1569,27 +1558,18 @@
       <c r="AF12"/>
       <c r="AG12"/>
       <c r="AH12"/>
-      <c r="AI12"/>
-      <c r="AJ12"/>
-      <c r="AK12"/>
-      <c r="AL12"/>
-      <c r="AM12"/>
-      <c r="AN12"/>
-      <c r="AO12"/>
-      <c r="AP12"/>
-      <c r="AQ12"/>
-    </row>
-    <row r="13" spans="1:43" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="19" t="s">
+    </row>
+    <row r="13" spans="1:34" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="B13" s="20"/>
-      <c r="C13" s="20"/>
-      <c r="D13" s="20"/>
-      <c r="E13" s="20"/>
-      <c r="F13" s="20"/>
-      <c r="G13" s="20"/>
-      <c r="H13" s="21"/>
+      <c r="B13" s="39"/>
+      <c r="C13" s="39"/>
+      <c r="D13" s="39"/>
+      <c r="E13" s="39"/>
+      <c r="F13" s="39"/>
+      <c r="G13" s="39"/>
+      <c r="H13" s="40"/>
       <c r="I13"/>
       <c r="J13"/>
       <c r="K13"/>
@@ -1616,29 +1596,20 @@
       <c r="AF13"/>
       <c r="AG13"/>
       <c r="AH13"/>
-      <c r="AI13"/>
-      <c r="AJ13"/>
-      <c r="AK13"/>
-      <c r="AL13"/>
-      <c r="AM13"/>
-      <c r="AN13"/>
-      <c r="AO13"/>
-      <c r="AP13"/>
-      <c r="AQ13"/>
-    </row>
-    <row r="14" spans="1:43" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="34" t="s">
-        <v>29</v>
-      </c>
-      <c r="B14" s="45" t="s">
+    </row>
+    <row r="14" spans="1:34" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="24" t="s">
+        <v>35</v>
+      </c>
+      <c r="B14" s="24" t="s">
         <v>33</v>
       </c>
-      <c r="C14" s="51"/>
-      <c r="D14" s="51"/>
-      <c r="E14" s="51"/>
-      <c r="F14" s="51"/>
-      <c r="G14" s="51"/>
-      <c r="H14" s="56"/>
+      <c r="C14" s="29"/>
+      <c r="D14" s="29"/>
+      <c r="E14" s="29"/>
+      <c r="F14" s="29"/>
+      <c r="G14" s="29"/>
+      <c r="H14" s="29"/>
       <c r="I14"/>
       <c r="J14"/>
       <c r="K14"/>
@@ -1665,25 +1636,16 @@
       <c r="AF14"/>
       <c r="AG14"/>
       <c r="AH14"/>
-      <c r="AI14"/>
-      <c r="AJ14"/>
-      <c r="AK14"/>
-      <c r="AL14"/>
-      <c r="AM14"/>
-      <c r="AN14"/>
-      <c r="AO14"/>
-      <c r="AP14"/>
-      <c r="AQ14"/>
-    </row>
-    <row r="15" spans="1:43" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="35"/>
-      <c r="B15" s="36"/>
-      <c r="C15" s="54"/>
-      <c r="D15" s="54"/>
-      <c r="E15" s="54"/>
-      <c r="F15" s="54"/>
-      <c r="G15" s="54"/>
-      <c r="H15" s="55"/>
+    </row>
+    <row r="15" spans="1:34" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="25"/>
+      <c r="B15" s="28"/>
+      <c r="C15" s="13"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="13"/>
+      <c r="F15" s="13"/>
+      <c r="G15" s="13"/>
+      <c r="H15" s="13"/>
       <c r="I15"/>
       <c r="J15"/>
       <c r="K15"/>
@@ -1710,27 +1672,20 @@
       <c r="AF15"/>
       <c r="AG15"/>
       <c r="AH15"/>
-      <c r="AI15"/>
-      <c r="AJ15"/>
-      <c r="AK15"/>
-      <c r="AL15"/>
-      <c r="AM15"/>
-      <c r="AN15"/>
-      <c r="AO15"/>
-      <c r="AP15"/>
-      <c r="AQ15"/>
-    </row>
-    <row r="16" spans="1:43" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="B16" s="20"/>
-      <c r="C16" s="20"/>
-      <c r="D16" s="20"/>
-      <c r="E16" s="20"/>
-      <c r="F16" s="20"/>
-      <c r="G16" s="20"/>
-      <c r="H16" s="21"/>
+    </row>
+    <row r="16" spans="1:34" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="26" t="s">
+        <v>32</v>
+      </c>
+      <c r="B16" s="26" t="s">
+        <v>34</v>
+      </c>
+      <c r="C16" s="13"/>
+      <c r="D16" s="13"/>
+      <c r="E16" s="13"/>
+      <c r="F16" s="13"/>
+      <c r="G16" s="13"/>
+      <c r="H16" s="13"/>
       <c r="I16"/>
       <c r="J16"/>
       <c r="K16"/>
@@ -1757,29 +1712,16 @@
       <c r="AF16"/>
       <c r="AG16"/>
       <c r="AH16"/>
-      <c r="AI16"/>
-      <c r="AJ16"/>
-      <c r="AK16"/>
-      <c r="AL16"/>
-      <c r="AM16"/>
-      <c r="AN16"/>
-      <c r="AO16"/>
-      <c r="AP16"/>
-      <c r="AQ16"/>
-    </row>
-    <row r="17" spans="1:43" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="34" t="s">
-        <v>30</v>
-      </c>
-      <c r="B17" s="45" t="s">
-        <v>34</v>
-      </c>
-      <c r="C17" s="51"/>
-      <c r="D17" s="51"/>
-      <c r="E17" s="51"/>
-      <c r="F17" s="51"/>
-      <c r="G17" s="51"/>
-      <c r="H17" s="56"/>
+    </row>
+    <row r="17" spans="1:34" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="27"/>
+      <c r="B17" s="27"/>
+      <c r="C17" s="14"/>
+      <c r="D17" s="14"/>
+      <c r="E17" s="14"/>
+      <c r="F17" s="14"/>
+      <c r="G17" s="14"/>
+      <c r="H17" s="14"/>
       <c r="I17"/>
       <c r="J17"/>
       <c r="K17"/>
@@ -1806,25 +1748,18 @@
       <c r="AF17"/>
       <c r="AG17"/>
       <c r="AH17"/>
-      <c r="AI17"/>
-      <c r="AJ17"/>
-      <c r="AK17"/>
-      <c r="AL17"/>
-      <c r="AM17"/>
-      <c r="AN17"/>
-      <c r="AO17"/>
-      <c r="AP17"/>
-      <c r="AQ17"/>
-    </row>
-    <row r="18" spans="1:43" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="35"/>
-      <c r="B18" s="36"/>
-      <c r="C18" s="54"/>
-      <c r="D18" s="54"/>
-      <c r="E18" s="54"/>
-      <c r="F18" s="54"/>
-      <c r="G18" s="54"/>
-      <c r="H18" s="55"/>
+    </row>
+    <row r="18" spans="1:34" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="21" t="s">
+        <v>22</v>
+      </c>
+      <c r="B18" s="22"/>
+      <c r="C18" s="22"/>
+      <c r="D18" s="22"/>
+      <c r="E18" s="22"/>
+      <c r="F18" s="22"/>
+      <c r="G18" s="22"/>
+      <c r="H18" s="23"/>
       <c r="I18"/>
       <c r="J18"/>
       <c r="K18"/>
@@ -1851,29 +1786,20 @@
       <c r="AF18"/>
       <c r="AG18"/>
       <c r="AH18"/>
-      <c r="AI18"/>
-      <c r="AJ18"/>
-      <c r="AK18"/>
-      <c r="AL18"/>
-      <c r="AM18"/>
-      <c r="AN18"/>
-      <c r="AO18"/>
-      <c r="AP18"/>
-      <c r="AQ18"/>
-    </row>
-    <row r="19" spans="1:43" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="34" t="s">
+    </row>
+    <row r="19" spans="1:34" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="19" t="s">
+        <v>29</v>
+      </c>
+      <c r="B19" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="B19" s="48" t="s">
-        <v>35</v>
-      </c>
-      <c r="C19" s="51"/>
-      <c r="D19" s="51"/>
-      <c r="E19" s="51"/>
-      <c r="F19" s="51"/>
-      <c r="G19" s="51"/>
-      <c r="H19" s="56"/>
+      <c r="C19" s="15"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="15"/>
+      <c r="F19" s="15"/>
+      <c r="G19" s="15"/>
+      <c r="H19" s="30"/>
       <c r="I19"/>
       <c r="J19"/>
       <c r="K19"/>
@@ -1900,25 +1826,16 @@
       <c r="AF19"/>
       <c r="AG19"/>
       <c r="AH19"/>
-      <c r="AI19"/>
-      <c r="AJ19"/>
-      <c r="AK19"/>
-      <c r="AL19"/>
-      <c r="AM19"/>
-      <c r="AN19"/>
-      <c r="AO19"/>
-      <c r="AP19"/>
-      <c r="AQ19"/>
-    </row>
-    <row r="20" spans="1:43" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="35"/>
-      <c r="B20" s="36"/>
-      <c r="C20" s="54"/>
-      <c r="D20" s="54"/>
-      <c r="E20" s="54"/>
-      <c r="F20" s="54"/>
-      <c r="G20" s="54"/>
-      <c r="H20" s="55"/>
+    </row>
+    <row r="20" spans="1:34" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="20"/>
+      <c r="B20" s="18"/>
+      <c r="C20" s="16"/>
+      <c r="D20" s="16"/>
+      <c r="E20" s="16"/>
+      <c r="F20" s="16"/>
+      <c r="G20" s="16"/>
+      <c r="H20" s="31"/>
       <c r="I20"/>
       <c r="J20"/>
       <c r="K20"/>
@@ -1945,25 +1862,8 @@
       <c r="AF20"/>
       <c r="AG20"/>
       <c r="AH20"/>
-      <c r="AI20"/>
-      <c r="AJ20"/>
-      <c r="AK20"/>
-      <c r="AL20"/>
-      <c r="AM20"/>
-      <c r="AN20"/>
-      <c r="AO20"/>
-      <c r="AP20"/>
-      <c r="AQ20"/>
-    </row>
-    <row r="21" spans="1:43" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21"/>
-      <c r="B21"/>
-      <c r="C21"/>
-      <c r="D21"/>
-      <c r="E21"/>
-      <c r="F21"/>
-      <c r="G21"/>
-      <c r="H21"/>
+    </row>
+    <row r="21" spans="1:34" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="I21"/>
       <c r="J21"/>
       <c r="K21"/>
@@ -1990,25 +1890,8 @@
       <c r="AF21"/>
       <c r="AG21"/>
       <c r="AH21"/>
-      <c r="AI21"/>
-      <c r="AJ21"/>
-      <c r="AK21"/>
-      <c r="AL21"/>
-      <c r="AM21"/>
-      <c r="AN21"/>
-      <c r="AO21"/>
-      <c r="AP21"/>
-      <c r="AQ21"/>
-    </row>
-    <row r="22" spans="1:43" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22"/>
-      <c r="B22"/>
-      <c r="C22"/>
-      <c r="D22"/>
-      <c r="E22"/>
-      <c r="F22"/>
-      <c r="G22"/>
-      <c r="H22"/>
+    </row>
+    <row r="22" spans="1:34" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="I22"/>
       <c r="J22"/>
       <c r="K22"/>
@@ -2035,17 +1918,8 @@
       <c r="AF22"/>
       <c r="AG22"/>
       <c r="AH22"/>
-      <c r="AI22"/>
-      <c r="AJ22"/>
-      <c r="AK22"/>
-      <c r="AL22"/>
-      <c r="AM22"/>
-      <c r="AN22"/>
-      <c r="AO22"/>
-      <c r="AP22"/>
-      <c r="AQ22"/>
-    </row>
-    <row r="23" spans="1:43" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="23" spans="1:34" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23"/>
       <c r="B23"/>
       <c r="C23"/>
@@ -2080,25 +1954,16 @@
       <c r="AF23"/>
       <c r="AG23"/>
       <c r="AH23"/>
-      <c r="AI23"/>
-      <c r="AJ23"/>
-      <c r="AK23"/>
-      <c r="AL23"/>
-      <c r="AM23"/>
-      <c r="AN23"/>
-      <c r="AO23"/>
-      <c r="AP23"/>
-      <c r="AQ23"/>
-    </row>
-    <row r="24" spans="1:43" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="10"/>
-      <c r="B24" s="11"/>
-      <c r="C24" s="12"/>
-      <c r="D24" s="12"/>
-      <c r="E24" s="12"/>
-      <c r="F24" s="12"/>
-      <c r="G24" s="12"/>
-      <c r="H24" s="12"/>
+    </row>
+    <row r="24" spans="1:34" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24"/>
+      <c r="B24"/>
+      <c r="C24"/>
+      <c r="D24"/>
+      <c r="E24"/>
+      <c r="F24"/>
+      <c r="G24"/>
+      <c r="H24"/>
       <c r="I24"/>
       <c r="J24"/>
       <c r="K24"/>
@@ -2125,17 +1990,8 @@
       <c r="AF24"/>
       <c r="AG24"/>
       <c r="AH24"/>
-      <c r="AI24"/>
-      <c r="AJ24"/>
-      <c r="AK24"/>
-      <c r="AL24"/>
-      <c r="AM24"/>
-      <c r="AN24"/>
-      <c r="AO24"/>
-      <c r="AP24"/>
-      <c r="AQ24"/>
-    </row>
-    <row r="25" spans="1:43" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="25" spans="1:34" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25"/>
       <c r="B25"/>
       <c r="C25"/>
@@ -2170,25 +2026,16 @@
       <c r="AF25"/>
       <c r="AG25"/>
       <c r="AH25"/>
-      <c r="AI25"/>
-      <c r="AJ25"/>
-      <c r="AK25"/>
-      <c r="AL25"/>
-      <c r="AM25"/>
-      <c r="AN25"/>
-      <c r="AO25"/>
-      <c r="AP25"/>
-      <c r="AQ25"/>
-    </row>
-    <row r="26" spans="1:43" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26"/>
-      <c r="B26"/>
-      <c r="C26"/>
-      <c r="D26"/>
-      <c r="E26"/>
-      <c r="F26"/>
-      <c r="G26"/>
-      <c r="H26"/>
+    </row>
+    <row r="26" spans="1:34" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="10"/>
+      <c r="B26" s="11"/>
+      <c r="C26" s="12"/>
+      <c r="D26" s="12"/>
+      <c r="E26" s="12"/>
+      <c r="F26" s="12"/>
+      <c r="G26" s="12"/>
+      <c r="H26" s="12"/>
       <c r="I26"/>
       <c r="J26"/>
       <c r="K26"/>
@@ -2215,17 +2062,8 @@
       <c r="AF26"/>
       <c r="AG26"/>
       <c r="AH26"/>
-      <c r="AI26"/>
-      <c r="AJ26"/>
-      <c r="AK26"/>
-      <c r="AL26"/>
-      <c r="AM26"/>
-      <c r="AN26"/>
-      <c r="AO26"/>
-      <c r="AP26"/>
-      <c r="AQ26"/>
-    </row>
-    <row r="27" spans="1:43" s="7" customFormat="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="27" spans="1:34" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27"/>
       <c r="B27"/>
       <c r="C27"/>
@@ -2260,17 +2098,8 @@
       <c r="AF27"/>
       <c r="AG27"/>
       <c r="AH27"/>
-      <c r="AI27"/>
-      <c r="AJ27"/>
-      <c r="AK27"/>
-      <c r="AL27"/>
-      <c r="AM27"/>
-      <c r="AN27"/>
-      <c r="AO27"/>
-      <c r="AP27"/>
-      <c r="AQ27"/>
-    </row>
-    <row r="28" spans="1:43" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="28" spans="1:34" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28"/>
       <c r="B28"/>
       <c r="C28"/>
@@ -2305,17 +2134,8 @@
       <c r="AF28"/>
       <c r="AG28"/>
       <c r="AH28"/>
-      <c r="AI28"/>
-      <c r="AJ28"/>
-      <c r="AK28"/>
-      <c r="AL28"/>
-      <c r="AM28"/>
-      <c r="AN28"/>
-      <c r="AO28"/>
-      <c r="AP28"/>
-      <c r="AQ28"/>
-    </row>
-    <row r="29" spans="1:43" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="29" spans="1:34" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A29"/>
       <c r="B29"/>
       <c r="C29"/>
@@ -2350,17 +2170,8 @@
       <c r="AF29"/>
       <c r="AG29"/>
       <c r="AH29"/>
-      <c r="AI29"/>
-      <c r="AJ29"/>
-      <c r="AK29"/>
-      <c r="AL29"/>
-      <c r="AM29"/>
-      <c r="AN29"/>
-      <c r="AO29"/>
-      <c r="AP29"/>
-      <c r="AQ29"/>
-    </row>
-    <row r="30" spans="1:43" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="30" spans="1:34" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30"/>
       <c r="B30"/>
       <c r="C30"/>
@@ -2395,17 +2206,8 @@
       <c r="AF30"/>
       <c r="AG30"/>
       <c r="AH30"/>
-      <c r="AI30"/>
-      <c r="AJ30"/>
-      <c r="AK30"/>
-      <c r="AL30"/>
-      <c r="AM30"/>
-      <c r="AN30"/>
-      <c r="AO30"/>
-      <c r="AP30"/>
-      <c r="AQ30"/>
-    </row>
-    <row r="31" spans="1:43" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="31" spans="1:34" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31"/>
       <c r="B31"/>
       <c r="C31"/>
@@ -2440,17 +2242,8 @@
       <c r="AF31"/>
       <c r="AG31"/>
       <c r="AH31"/>
-      <c r="AI31"/>
-      <c r="AJ31"/>
-      <c r="AK31"/>
-      <c r="AL31"/>
-      <c r="AM31"/>
-      <c r="AN31"/>
-      <c r="AO31"/>
-      <c r="AP31"/>
-      <c r="AQ31"/>
-    </row>
-    <row r="32" spans="1:43" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="32" spans="1:34" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32"/>
       <c r="B32"/>
       <c r="C32"/>
@@ -2478,8 +2271,15 @@
       <c r="Y32"/>
       <c r="Z32"/>
       <c r="AA32"/>
-    </row>
-    <row r="33" spans="1:43" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AB32"/>
+      <c r="AC32"/>
+      <c r="AD32"/>
+      <c r="AE32"/>
+      <c r="AF32"/>
+      <c r="AG32"/>
+      <c r="AH32"/>
+    </row>
+    <row r="33" spans="1:34" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33"/>
       <c r="B33"/>
       <c r="C33"/>
@@ -2507,8 +2307,15 @@
       <c r="Y33"/>
       <c r="Z33"/>
       <c r="AA33"/>
-    </row>
-    <row r="34" spans="1:43" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AB33"/>
+      <c r="AC33"/>
+      <c r="AD33"/>
+      <c r="AE33"/>
+      <c r="AF33"/>
+      <c r="AG33"/>
+      <c r="AH33"/>
+    </row>
+    <row r="34" spans="1:34" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34"/>
       <c r="B34"/>
       <c r="C34"/>
@@ -2527,17 +2334,8 @@
       <c r="P34"/>
       <c r="Q34"/>
       <c r="R34"/>
-      <c r="S34"/>
-      <c r="T34"/>
-      <c r="U34"/>
-      <c r="V34"/>
-      <c r="W34"/>
-      <c r="X34"/>
-      <c r="Y34"/>
-      <c r="Z34"/>
-      <c r="AA34"/>
-    </row>
-    <row r="35" spans="1:43" s="7" customFormat="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="35" spans="1:34" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35"/>
       <c r="B35"/>
       <c r="C35"/>
@@ -2556,45 +2354,74 @@
       <c r="P35"/>
       <c r="Q35"/>
       <c r="R35"/>
-      <c r="S35"/>
-      <c r="T35"/>
-      <c r="U35"/>
-      <c r="V35"/>
-      <c r="W35"/>
-      <c r="X35"/>
-      <c r="Y35"/>
-      <c r="Z35"/>
-      <c r="AA35"/>
-      <c r="AB35"/>
-      <c r="AC35"/>
-      <c r="AD35"/>
-      <c r="AE35"/>
-      <c r="AF35"/>
-      <c r="AG35"/>
-      <c r="AH35"/>
-      <c r="AI35"/>
-      <c r="AJ35"/>
-      <c r="AK35"/>
-      <c r="AL35"/>
-      <c r="AM35"/>
-      <c r="AN35"/>
-      <c r="AO35"/>
-      <c r="AP35"/>
-      <c r="AQ35"/>
-    </row>
-    <row r="36" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="37" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="38" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="39" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="40" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="41" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="42" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="43" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="44" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="45" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="46" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="47" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="48" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
+    </row>
+    <row r="36" spans="1:34" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36"/>
+      <c r="B36"/>
+      <c r="C36"/>
+      <c r="D36"/>
+      <c r="E36"/>
+      <c r="F36"/>
+      <c r="G36"/>
+      <c r="H36"/>
+      <c r="I36"/>
+      <c r="J36"/>
+      <c r="K36"/>
+      <c r="L36"/>
+      <c r="M36"/>
+      <c r="N36"/>
+      <c r="O36"/>
+      <c r="P36"/>
+      <c r="Q36"/>
+      <c r="R36"/>
+    </row>
+    <row r="37" spans="1:34" s="7" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A37"/>
+      <c r="B37"/>
+      <c r="C37"/>
+      <c r="D37"/>
+      <c r="E37"/>
+      <c r="F37"/>
+      <c r="G37"/>
+      <c r="H37"/>
+      <c r="I37"/>
+      <c r="J37"/>
+      <c r="K37"/>
+      <c r="L37"/>
+      <c r="M37"/>
+      <c r="N37"/>
+      <c r="O37"/>
+      <c r="P37"/>
+      <c r="Q37"/>
+      <c r="R37"/>
+      <c r="S37"/>
+      <c r="T37"/>
+      <c r="U37"/>
+      <c r="V37"/>
+      <c r="W37"/>
+      <c r="X37"/>
+      <c r="Y37"/>
+      <c r="Z37"/>
+      <c r="AA37"/>
+      <c r="AB37"/>
+      <c r="AC37"/>
+      <c r="AD37"/>
+      <c r="AE37"/>
+      <c r="AF37"/>
+      <c r="AG37"/>
+      <c r="AH37"/>
+    </row>
+    <row r="38" spans="1:34" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="39" spans="1:34" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="40" spans="1:34" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="41" spans="1:34" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="42" spans="1:34" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="43" spans="1:34" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="44" spans="1:34" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="45" spans="1:34" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="46" spans="1:34" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="47" spans="1:34" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="48" spans="1:34" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="49" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="50" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="51" customFormat="1" x14ac:dyDescent="0.2"/>
@@ -2617,26 +2444,8 @@
     <row r="68" spans="1:8" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="69" spans="1:8" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="70" spans="1:8" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="71" spans="1:8" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A71" s="1"/>
-      <c r="B71" s="1"/>
-      <c r="C71" s="1"/>
-      <c r="D71" s="1"/>
-      <c r="E71" s="1"/>
-      <c r="F71" s="1"/>
-      <c r="G71" s="1"/>
-      <c r="H71" s="1"/>
-    </row>
-    <row r="72" spans="1:8" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A72" s="1"/>
-      <c r="B72" s="1"/>
-      <c r="C72" s="1"/>
-      <c r="D72" s="1"/>
-      <c r="E72" s="1"/>
-      <c r="F72" s="1"/>
-      <c r="G72" s="1"/>
-      <c r="H72" s="1"/>
-    </row>
+    <row r="71" spans="1:8" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="72" spans="1:8" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="73" spans="1:8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A73" s="1"/>
       <c r="B73" s="1"/>
@@ -2727,24 +2536,40 @@
       <c r="G81" s="1"/>
       <c r="H81" s="1"/>
     </row>
+    <row r="82" spans="1:8" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A82" s="1"/>
+      <c r="B82" s="1"/>
+      <c r="C82" s="1"/>
+      <c r="D82" s="1"/>
+      <c r="E82" s="1"/>
+      <c r="F82" s="1"/>
+      <c r="G82" s="1"/>
+      <c r="H82" s="1"/>
+    </row>
+    <row r="83" spans="1:8" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A83" s="1"/>
+      <c r="B83" s="1"/>
+      <c r="C83" s="1"/>
+      <c r="D83" s="1"/>
+      <c r="E83" s="1"/>
+      <c r="F83" s="1"/>
+      <c r="G83" s="1"/>
+      <c r="H83" s="1"/>
+    </row>
   </sheetData>
   <mergeCells count="52">
-    <mergeCell ref="F17:F18"/>
-    <mergeCell ref="G17:G18"/>
-    <mergeCell ref="H17:H18"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="C19:C20"/>
-    <mergeCell ref="D19:D20"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="F19:F20"/>
-    <mergeCell ref="G19:G20"/>
-    <mergeCell ref="H19:H20"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="D17:D18"/>
-    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="H11:H12"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="A13:H13"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="A8:H8"/>
     <mergeCell ref="F9:F10"/>
     <mergeCell ref="G9:G10"/>
     <mergeCell ref="H9:H10"/>
@@ -2755,20 +2580,16 @@
     <mergeCell ref="E11:E12"/>
     <mergeCell ref="F11:F12"/>
     <mergeCell ref="G11:G12"/>
-    <mergeCell ref="H11:H12"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="A13:H13"/>
-    <mergeCell ref="A16:H16"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A5:H5"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="A8:H8"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="F3:H3"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="A18:H18"/>
     <mergeCell ref="A14:A15"/>
+    <mergeCell ref="A16:A17"/>
     <mergeCell ref="B14:B15"/>
     <mergeCell ref="C14:C15"/>
     <mergeCell ref="D14:D15"/>
@@ -2776,11 +2597,19 @@
     <mergeCell ref="F14:F15"/>
     <mergeCell ref="G14:G15"/>
     <mergeCell ref="H14:H15"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="F3:H3"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="D16:D17"/>
+    <mergeCell ref="H19:H20"/>
+    <mergeCell ref="E16:E17"/>
+    <mergeCell ref="F16:F17"/>
+    <mergeCell ref="G16:G17"/>
+    <mergeCell ref="H16:H17"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="G19:G20"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="D19:D20"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.19685039370078738" right="0.19685039370078738" top="0.19685039370078738" bottom="0.19685039370078738" header="0.51181102362204722" footer="0.51181102362204722"/>

</xml_diff>